<commit_message>
Finalize project documentation and figures
</commit_message>
<xml_diff>
--- a/Projet 3 - Checklist.xlsx
+++ b/Projet 3 - Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bdptenant-my.sharepoint.com/personal/r_dasilva_fr_motul_com/Documents/Bureau/data_scientist/project_3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="364" documentId="8_{ED160A35-4349-40D9-B442-4E161748A9D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BF06F18E-1BE5-4915-A9FC-132ECE960FC9}"/>
+  <xr:revisionPtr revIDLastSave="373" documentId="8_{ED160A35-4349-40D9-B442-4E161748A9D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B3A3A0D7-76F1-4DA3-B294-3646818B7E71}"/>
   <bookViews>
     <workbookView xWindow="-9315" yWindow="-14820" windowWidth="17280" windowHeight="8880" activeTab="4" xr2:uid="{B440E984-6FB6-48FF-8FAC-CDDF955D1CA9}"/>
   </bookViews>
@@ -3071,8 +3071,5 @@
     <hyperlink ref="C17" r:id="rId2" display="https://scikit-learn.org/stable/modules/generated/sklearn.model_selection.GridSearchCV.html" xr:uid="{CFB2E0C7-62E1-4E88-9B14-90296AB7E783}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <customProperties>
-    <customPr name="IbpWorksheetKeyString_GUID" r:id="rId3"/>
-  </customProperties>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Clean notebooks and improve pipeline documentation
</commit_message>
<xml_diff>
--- a/Projet 3 - Checklist.xlsx
+++ b/Projet 3 - Checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bdptenant-my.sharepoint.com/personal/r_dasilva_fr_motul_com/Documents/Bureau/data_scientist/project_3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="373" documentId="8_{ED160A35-4349-40D9-B442-4E161748A9D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B3A3A0D7-76F1-4DA3-B294-3646818B7E71}"/>
+  <xr:revisionPtr revIDLastSave="379" documentId="8_{ED160A35-4349-40D9-B442-4E161748A9D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF622345-0AE3-400C-A900-5EE27705D478}"/>
   <bookViews>
-    <workbookView xWindow="-9315" yWindow="-14820" windowWidth="17280" windowHeight="8880" activeTab="4" xr2:uid="{B440E984-6FB6-48FF-8FAC-CDDF955D1CA9}"/>
+    <workbookView xWindow="-16035" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{B440E984-6FB6-48FF-8FAC-CDDF955D1CA9}"/>
   </bookViews>
   <sheets>
     <sheet name="E1" sheetId="2" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="131">
   <si>
     <t>Prérequis </t>
   </si>
@@ -1828,7 +1828,7 @@
       </c>
       <c r="F16" s="2"/>
     </row>
-    <row r="17" spans="2:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B17" s="10" t="s">
         <v>11</v>
       </c>
@@ -1918,8 +1918,12 @@
       <c r="D4" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="13"/>
-      <c r="F4" s="13"/>
+      <c r="E4" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="5" spans="2:6" ht="156" x14ac:dyDescent="0.3">
       <c r="B5" s="18" t="s">
@@ -1949,7 +1953,7 @@
       <c r="E6" s="13"/>
       <c r="F6" s="13"/>
     </row>
-    <row r="7" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:6" s="3" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B7" s="21" t="s">
         <v>4</v>
       </c>
@@ -1962,9 +1966,11 @@
       <c r="E7" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="F7" s="13"/>
-    </row>
-    <row r="8" spans="2:6" s="3" customFormat="1" ht="24" x14ac:dyDescent="0.3">
+      <c r="F7" s="13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" s="3" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B8" s="21" t="s">
         <v>4</v>
       </c>
@@ -1977,7 +1983,9 @@
       <c r="E8" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="F8" s="13"/>
+      <c r="F8" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="9" spans="2:6" s="3" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B9" s="21" t="s">
@@ -1988,7 +1996,9 @@
       </c>
       <c r="D9" s="14"/>
       <c r="E9" s="13"/>
-      <c r="F9" s="13"/>
+      <c r="F9" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="10" spans="2:6" s="3" customFormat="1" ht="46.8" x14ac:dyDescent="0.3">
       <c r="B10" s="21" t="s">
@@ -2003,7 +2013,9 @@
       <c r="E10" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="F10" s="13"/>
+      <c r="F10" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="11" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B11" s="21" t="s">
@@ -2018,7 +2030,9 @@
       <c r="E11" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="F11" s="13"/>
+      <c r="F11" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="12" spans="2:6" s="3" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B12" s="21" t="s">
@@ -2033,7 +2047,9 @@
       <c r="E12" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="F12" s="13"/>
+      <c r="F12" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.3">
       <c r="D13" s="14"/>
@@ -2058,6 +2074,9 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <customProperties>
+    <customPr name="IbpWorksheetKeyString_GUID" r:id="rId1"/>
+  </customProperties>
 </worksheet>
 </file>
 
@@ -2376,6 +2395,9 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <customProperties>
+    <customPr name="IbpWorksheetKeyString_GUID" r:id="rId1"/>
+  </customProperties>
 </worksheet>
 </file>
 
@@ -3071,5 +3093,8 @@
     <hyperlink ref="C17" r:id="rId2" display="https://scikit-learn.org/stable/modules/generated/sklearn.model_selection.GridSearchCV.html" xr:uid="{CFB2E0C7-62E1-4E88-9B14-90296AB7E783}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <customProperties>
+    <customPr name="IbpWorksheetKeyString_GUID" r:id="rId3"/>
+  </customProperties>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
refactor: update project after mentor feedback and complete review
</commit_message>
<xml_diff>
--- a/Projet 3 - Checklist.xlsx
+++ b/Projet 3 - Checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bdptenant-my.sharepoint.com/personal/r_dasilva_fr_motul_com/Documents/Bureau/data_scientist/project_3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="379" documentId="8_{ED160A35-4349-40D9-B442-4E161748A9D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF622345-0AE3-400C-A900-5EE27705D478}"/>
+  <xr:revisionPtr revIDLastSave="409" documentId="8_{ED160A35-4349-40D9-B442-4E161748A9D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{56473DD1-CCD8-41D4-8DA6-1B23CDE6FBCD}"/>
   <bookViews>
-    <workbookView xWindow="-16035" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{B440E984-6FB6-48FF-8FAC-CDDF955D1CA9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{B440E984-6FB6-48FF-8FAC-CDDF955D1CA9}"/>
   </bookViews>
   <sheets>
     <sheet name="E1" sheetId="2" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="131">
   <si>
     <t>Prérequis </t>
   </si>
@@ -425,9 +425,6 @@
     <t>&gt; -  Les valeurs extrêmes correspondent majoritairement à des bâtiments de grande taille et font partie de la variabilité naturelle du jeu de données. Elles sont donc conservées pour la modélisation.</t>
   </si>
   <si>
-    <t>ÉTAPE 4 : Preparez les features pour la modelisation</t>
-  </si>
-  <si>
     <t>ce qu'est une séparation train-test et ce qu'est une validation croisée ;</t>
   </si>
   <si>
@@ -816,6 +813,9 @@
   </si>
   <si>
     <t>Petite grille de test</t>
+  </si>
+  <si>
+    <t>ÉTAPE 4 : COMPAIRAISON SUPERVISEE</t>
   </si>
 </sst>
 </file>
@@ -1640,7 +1640,7 @@
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B4" s="33" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C4" s="31" t="s">
         <v>24</v>
@@ -1870,6 +1870,9 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <customProperties>
+    <customPr name="IbpWorksheetKeyString_GUID" r:id="rId1"/>
+  </customProperties>
 </worksheet>
 </file>
 
@@ -1953,7 +1956,7 @@
       <c r="E6" s="13"/>
       <c r="F6" s="13"/>
     </row>
-    <row r="7" spans="2:6" s="3" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B7" s="21" t="s">
         <v>4</v>
       </c>
@@ -1970,7 +1973,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="2:6" s="3" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:6" s="3" customFormat="1" ht="24" x14ac:dyDescent="0.3">
       <c r="B8" s="21" t="s">
         <v>4</v>
       </c>
@@ -1987,7 +1990,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="2:6" s="3" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B9" s="21" t="s">
         <v>4</v>
       </c>
@@ -2082,7 +2085,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A88BAC3-9941-4922-B957-2F2B13FDA549}">
-  <dimension ref="B2:F25"/>
+  <dimension ref="B2:F24"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="26.33203125" style="34" customWidth="1"/>
@@ -2107,6 +2110,10 @@
       </c>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B3" s="34" t="str">
+        <f>UPPER(C3)</f>
+        <v>ÉTAPE 3 : PREPAREZ LES FEATURES POUR LA MODELISATION</v>
+      </c>
       <c r="C3" s="17" t="s">
         <v>56</v>
       </c>
@@ -2124,8 +2131,12 @@
       <c r="D4" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="38"/>
-      <c r="F4" s="13"/>
+      <c r="E4" s="38" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B5" s="18" t="s">
@@ -2140,7 +2151,9 @@
       <c r="E5" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="F5" s="13"/>
+      <c r="F5" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="6" spans="2:6" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B6" s="18" t="s">
@@ -2150,15 +2163,23 @@
         <v>59</v>
       </c>
       <c r="D6" s="14"/>
-      <c r="E6" s="38"/>
-      <c r="F6" s="13"/>
+      <c r="E6" s="38" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B7" s="18"/>
       <c r="C7" s="19"/>
       <c r="D7" s="14"/>
-      <c r="E7" s="38"/>
-      <c r="F7" s="13"/>
+      <c r="E7" s="38" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B8" s="21" t="s">
@@ -2168,8 +2189,12 @@
         <v>44</v>
       </c>
       <c r="D8" s="6"/>
-      <c r="E8" s="38"/>
-      <c r="F8" s="13"/>
+      <c r="E8" s="38" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B9" s="21" t="s">
@@ -2184,7 +2209,9 @@
       <c r="E9" s="38" t="s">
         <v>35</v>
       </c>
-      <c r="F9" s="13"/>
+      <c r="F9" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B10" s="37" t="s">
@@ -2199,7 +2226,9 @@
       <c r="E10" s="38" t="s">
         <v>29</v>
       </c>
-      <c r="F10" s="13"/>
+      <c r="F10" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="11" spans="2:6" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B11" s="21" t="s">
@@ -2214,7 +2243,9 @@
       <c r="E11" s="38" t="s">
         <v>78</v>
       </c>
-      <c r="F11" s="13"/>
+      <c r="F11" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="12" spans="2:6" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B12" s="21" t="s">
@@ -2229,7 +2260,9 @@
       <c r="E12" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="F12" s="13"/>
+      <c r="F12" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B13" s="21" t="s">
@@ -2244,7 +2277,9 @@
       <c r="E13" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="F13" s="13"/>
+      <c r="F13" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="14" spans="2:6" ht="60" x14ac:dyDescent="0.3">
       <c r="B14" s="21" t="s">
@@ -2263,133 +2298,153 @@
         <v>40</v>
       </c>
     </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="C15" s="36"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="38"/>
-      <c r="F15" s="13"/>
-    </row>
-    <row r="16" spans="2:6" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:6" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="B15" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" s="36" t="s">
+        <v>60</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E15" s="38" t="s">
+        <v>79</v>
+      </c>
+      <c r="F15" s="13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B16" s="18" t="s">
         <v>4</v>
       </c>
       <c r="C16" s="36" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E16" s="38" t="s">
-        <v>79</v>
-      </c>
-      <c r="F16" s="13"/>
+      <c r="E16" s="39" t="s">
+        <v>76</v>
+      </c>
+      <c r="F16" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B17" s="18" t="s">
         <v>4</v>
       </c>
       <c r="C17" s="36" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E17" s="39" t="s">
-        <v>76</v>
-      </c>
-      <c r="F17" s="13"/>
-    </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="E17" s="38" t="s">
+        <v>77</v>
+      </c>
+      <c r="F17" s="13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B18" s="18" t="s">
         <v>4</v>
       </c>
       <c r="C18" s="36" t="s">
-        <v>62</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>16</v>
-      </c>
+        <v>63</v>
+      </c>
+      <c r="D18" s="6"/>
       <c r="E18" s="38" t="s">
-        <v>77</v>
-      </c>
-      <c r="F18" s="13"/>
+        <v>15</v>
+      </c>
+      <c r="F18" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="19" spans="2:6" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B19" s="18" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C19" s="36" t="s">
-        <v>63</v>
-      </c>
-      <c r="D19" s="6"/>
-      <c r="E19" s="38"/>
-      <c r="F19" s="13"/>
-    </row>
-    <row r="20" spans="2:6" ht="31.2" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E19" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F19" s="13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B20" s="18" t="s">
         <v>11</v>
       </c>
       <c r="C20" s="36" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D20" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E20" s="13"/>
-      <c r="F20" s="13"/>
-    </row>
-    <row r="21" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="E20" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F20" s="13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" s="3" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B21" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="36" t="s">
-        <v>65</v>
+      <c r="C21" s="20" t="s">
+        <v>66</v>
       </c>
       <c r="D21" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E21" s="13"/>
-      <c r="F21" s="13"/>
+      <c r="E21" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F21" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="22" spans="2:6" s="3" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B22" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="C22" s="20" t="s">
-        <v>66</v>
+      <c r="C22" s="23" t="s">
+        <v>50</v>
       </c>
       <c r="D22" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E22" s="13"/>
-      <c r="F22" s="13"/>
-    </row>
-    <row r="23" spans="2:6" s="3" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B23" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="C23" s="23" t="s">
-        <v>50</v>
-      </c>
-      <c r="D23" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E23" s="13"/>
-      <c r="F23" s="13"/>
+      <c r="E22" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F22" s="13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="D23" s="14"/>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.3">
       <c r="D24" s="14"/>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="D25" s="14"/>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="D4:D5 D16:D23">
+  <conditionalFormatting sqref="D4:D5">
     <cfRule type="cellIs" dxfId="4" priority="14" operator="equal">
       <formula>"P"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D8:D14">
+  <conditionalFormatting sqref="D8:D22">
     <cfRule type="cellIs" dxfId="3" priority="7" operator="equal">
       <formula>"P"</formula>
     </cfRule>
@@ -2429,7 +2484,7 @@
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.3">
       <c r="C3" s="17" t="s">
-        <v>80</v>
+        <v>130</v>
       </c>
       <c r="D3" s="12"/>
       <c r="E3" s="38"/>
@@ -2440,20 +2495,24 @@
         <v>0</v>
       </c>
       <c r="C4" s="36" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="38"/>
-      <c r="F4" s="13"/>
+      <c r="E4" s="38" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B5" s="18" t="s">
         <v>0</v>
       </c>
       <c r="C5" s="36" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D5" s="6" t="s">
         <v>16</v>
@@ -2461,107 +2520,141 @@
       <c r="E5" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="F5" s="13"/>
+      <c r="F5" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B6" s="18" t="s">
         <v>0</v>
       </c>
       <c r="C6" s="36" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D6" s="14"/>
-      <c r="E6" s="38"/>
-      <c r="F6" s="13"/>
+      <c r="E6" s="38" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B7" s="18" t="s">
         <v>0</v>
       </c>
       <c r="C7" s="36" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D7" s="14"/>
-      <c r="E7" s="38"/>
-      <c r="F7" s="13"/>
+      <c r="E7" s="38" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B8" s="18"/>
       <c r="C8" s="36"/>
       <c r="D8" s="14"/>
-      <c r="E8" s="38"/>
-      <c r="F8" s="13"/>
+      <c r="E8" s="38" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B9" s="18" t="s">
         <v>2</v>
       </c>
       <c r="C9" s="36" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E9" s="38"/>
-      <c r="F9" s="13"/>
+      <c r="E9" s="38" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B10" s="21"/>
       <c r="C10" s="36"/>
       <c r="D10" s="6"/>
-      <c r="E10" s="38"/>
-      <c r="F10" s="13"/>
+      <c r="E10" s="38" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B11" s="21" t="s">
         <v>67</v>
       </c>
       <c r="C11" s="36" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D11" s="6"/>
-      <c r="E11" s="38"/>
-      <c r="F11" s="13"/>
+      <c r="E11" s="38" t="s">
+        <v>15</v>
+      </c>
+      <c r="F11" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B12" s="37" t="s">
         <v>67</v>
       </c>
       <c r="C12" s="36" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>16</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="F12" s="13"/>
+        <v>105</v>
+      </c>
+      <c r="F12" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="13" spans="2:6" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B13" s="21" t="s">
         <v>67</v>
       </c>
       <c r="C13" s="36" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D13" s="6"/>
+      <c r="E13" s="41" t="s">
+        <v>15</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B14" s="21" t="s">
         <v>67</v>
       </c>
       <c r="C14" s="36" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>16</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F14" s="13" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.3">
@@ -2569,31 +2662,33 @@
         <v>67</v>
       </c>
       <c r="C15" s="36" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>16</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="F15" s="13"/>
+        <v>108</v>
+      </c>
+      <c r="F15" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B16" s="21" t="s">
         <v>67</v>
       </c>
       <c r="C16" s="36" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>16</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.3">
@@ -2601,29 +2696,33 @@
         <v>67</v>
       </c>
       <c r="C17" s="36" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E17" s="38"/>
-      <c r="F17" s="13"/>
+      <c r="E17" s="38" t="s">
+        <v>15</v>
+      </c>
+      <c r="F17" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B18" s="21" t="s">
         <v>67</v>
       </c>
       <c r="C18" s="36" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>16</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F18" s="13" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.3">
@@ -2631,175 +2730,222 @@
         <v>67</v>
       </c>
       <c r="C19" s="36" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D19" s="6" t="s">
         <v>16</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>110</v>
+        <v>109</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B20" s="21"/>
       <c r="C20" s="36"/>
       <c r="D20" s="6"/>
-      <c r="E20" s="38"/>
-      <c r="F20" s="13"/>
+      <c r="E20" s="38" t="s">
+        <v>15</v>
+      </c>
+      <c r="F20" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="21" spans="2:6" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B21" s="18" t="s">
         <v>4</v>
       </c>
       <c r="C21" s="36" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D21" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E21" s="38"/>
-      <c r="F21" s="13"/>
+      <c r="E21" s="38" t="s">
+        <v>15</v>
+      </c>
+      <c r="F21" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="22" spans="2:6" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B22" s="18" t="s">
         <v>4</v>
       </c>
       <c r="C22" s="36" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D22" s="6"/>
-      <c r="E22" s="39"/>
-      <c r="F22" s="13"/>
+      <c r="E22" s="39" t="s">
+        <v>15</v>
+      </c>
+      <c r="F22" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B23" s="18" t="s">
         <v>4</v>
       </c>
       <c r="C23" s="36" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>16</v>
       </c>
       <c r="E23" s="40" t="s">
-        <v>111</v>
-      </c>
-      <c r="F23" s="13"/>
+        <v>110</v>
+      </c>
+      <c r="F23" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B24" s="18" t="s">
         <v>4</v>
       </c>
       <c r="C24" s="36" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D24" s="6" t="s">
         <v>16</v>
       </c>
       <c r="E24" s="40" t="s">
-        <v>112</v>
-      </c>
-      <c r="F24" s="13"/>
+        <v>111</v>
+      </c>
+      <c r="F24" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B25" s="18" t="s">
         <v>4</v>
       </c>
       <c r="C25" s="36" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D25" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E25" s="13"/>
-      <c r="F25" s="13"/>
+      <c r="E25" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F25" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="26" spans="2:6" s="3" customFormat="1" ht="46.8" x14ac:dyDescent="0.3">
       <c r="B26" s="18" t="s">
         <v>4</v>
       </c>
       <c r="C26" s="36" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D26" s="6" t="s">
         <v>16</v>
       </c>
       <c r="E26" s="40" t="s">
-        <v>113</v>
-      </c>
-      <c r="F26" s="13"/>
+        <v>112</v>
+      </c>
+      <c r="F26" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="27" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B27" s="18"/>
       <c r="C27" s="36"/>
       <c r="D27" s="14"/>
-      <c r="E27" s="13"/>
-      <c r="F27" s="13"/>
+      <c r="E27" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F27" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="28" spans="2:6" s="3" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B28" s="18" t="s">
         <v>11</v>
       </c>
       <c r="C28" s="36" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D28" s="6" t="s">
         <v>16</v>
       </c>
       <c r="E28" s="40" t="s">
-        <v>112</v>
-      </c>
-      <c r="F28" s="13"/>
+        <v>111</v>
+      </c>
+      <c r="F28" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="29" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B29" s="18" t="s">
         <v>14</v>
       </c>
       <c r="C29" s="36" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D29" s="6"/>
-      <c r="E29" s="40"/>
-      <c r="F29" s="13"/>
+      <c r="E29" s="40" t="s">
+        <v>15</v>
+      </c>
+      <c r="F29" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="30" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B30" s="18" t="s">
         <v>14</v>
       </c>
       <c r="C30" s="36" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D30" s="43" t="s">
-        <v>114</v>
-      </c>
-      <c r="E30" s="40"/>
-      <c r="F30" s="13"/>
+        <v>113</v>
+      </c>
+      <c r="E30" s="40" t="s">
+        <v>15</v>
+      </c>
+      <c r="F30" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="31" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B31" s="18" t="s">
         <v>14</v>
       </c>
       <c r="C31" s="36" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D31" s="43" t="s">
         <v>15</v>
       </c>
-      <c r="E31" s="40"/>
-      <c r="F31" s="13"/>
+      <c r="E31" s="40" t="s">
+        <v>15</v>
+      </c>
+      <c r="F31" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="32" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B32" s="18" t="s">
         <v>14</v>
       </c>
       <c r="C32" s="36" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D32" s="43" t="s">
         <v>15</v>
       </c>
-      <c r="E32" s="40"/>
-      <c r="F32" s="13"/>
+      <c r="E32" s="40" t="s">
+        <v>15</v>
+      </c>
+      <c r="F32" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="33" spans="2:6" s="3" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B33" s="34"/>
@@ -2845,7 +2991,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C49E4A0-6108-4A9F-A245-2E48F697262D}">
-  <dimension ref="B2:F24"/>
+  <dimension ref="B2:F22"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="26.33203125" style="34" customWidth="1"/>
@@ -2871,7 +3017,7 @@
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.3">
       <c r="C3" s="17" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D3" s="12"/>
       <c r="E3" s="38"/>
@@ -2882,95 +3028,119 @@
         <v>0</v>
       </c>
       <c r="C4" s="36" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="38"/>
-      <c r="F4" s="13"/>
+      <c r="E4" s="38" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B5" s="18" t="s">
         <v>2</v>
       </c>
       <c r="C5" s="36" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D5" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="38"/>
-      <c r="F5" s="13"/>
+      <c r="E5" s="38" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B6" s="37" t="s">
         <v>67</v>
       </c>
       <c r="C6" s="36" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>16</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="F6" s="13"/>
+        <v>105</v>
+      </c>
+      <c r="F6" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="7" spans="2:6" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B7" s="21" t="s">
         <v>67</v>
       </c>
       <c r="C7" s="36" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>16</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B8" s="21"/>
-      <c r="C8" s="36"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="38"/>
-      <c r="F8" s="13"/>
+        <v>106</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="B8" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="36" t="s">
+        <v>117</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="F8" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="9" spans="2:6" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B9" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="36" t="s">
-        <v>118</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>16</v>
-      </c>
+      <c r="C9" s="44" t="s">
+        <v>127</v>
+      </c>
+      <c r="D9" s="6"/>
       <c r="E9" s="38" t="s">
         <v>129</v>
       </c>
-      <c r="F9" s="13"/>
+      <c r="F9" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="10" spans="2:6" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B10" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="C10" s="44" t="s">
-        <v>128</v>
-      </c>
-      <c r="D10" s="6"/>
-      <c r="E10" s="38" t="s">
-        <v>130</v>
-      </c>
-      <c r="F10" s="13"/>
-    </row>
-    <row r="11" spans="2:6" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="C10" s="36" t="s">
+        <v>118</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E10" s="40" t="s">
+        <v>110</v>
+      </c>
+      <c r="F10" s="13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B11" s="18" t="s">
         <v>4</v>
       </c>
@@ -2983,11 +3153,13 @@
       <c r="E11" s="40" t="s">
         <v>111</v>
       </c>
-      <c r="F11" s="13"/>
-    </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="F11" s="13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" s="3" customFormat="1" ht="46.8" x14ac:dyDescent="0.3">
       <c r="B12" s="18" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C12" s="36" t="s">
         <v>120</v>
@@ -2996,105 +3168,94 @@
         <v>16</v>
       </c>
       <c r="E12" s="40" t="s">
-        <v>112</v>
-      </c>
-      <c r="F12" s="13"/>
-    </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B13" s="18"/>
-      <c r="C13" s="36"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="13"/>
-    </row>
-    <row r="14" spans="2:6" s="3" customFormat="1" ht="46.8" x14ac:dyDescent="0.3">
+        <v>111</v>
+      </c>
+      <c r="F12" s="13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" s="3" customFormat="1" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="B13" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="C13" s="36" t="s">
+        <v>121</v>
+      </c>
+      <c r="D13" s="42"/>
+      <c r="E13" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F13" s="13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B14" s="18" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C14" s="36" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E14" s="40" t="s">
-        <v>112</v>
-      </c>
-      <c r="F14" s="13"/>
-    </row>
-    <row r="15" spans="2:6" s="3" customFormat="1" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="E14" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F14" s="13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B15" s="18" t="s">
         <v>14</v>
       </c>
       <c r="C15" s="36" t="s">
-        <v>122</v>
-      </c>
-      <c r="D15" s="42"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
-    </row>
-    <row r="16" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C16" s="36" t="s">
         <v>123</v>
       </c>
-      <c r="D16" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E16" s="13"/>
-      <c r="F16" s="13"/>
-    </row>
-    <row r="17" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C17" s="36" t="s">
-        <v>124</v>
-      </c>
-      <c r="D17" s="42" t="s">
-        <v>15</v>
-      </c>
-      <c r="E17" s="13"/>
-      <c r="F17" s="13"/>
-    </row>
-    <row r="18" spans="2:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="D15" s="42" t="s">
+        <v>15</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F15" s="13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C16" s="34"/>
+      <c r="D16" s="14"/>
+    </row>
+    <row r="17" spans="3:4" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C17" s="34"/>
+      <c r="D17" s="14"/>
+    </row>
+    <row r="18" spans="3:4" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C18" s="34"/>
-      <c r="D18" s="14"/>
-    </row>
-    <row r="19" spans="2:6" ht="14.4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="19" spans="3:4" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C19" s="34"/>
-      <c r="D19" s="14"/>
-    </row>
-    <row r="20" spans="2:6" ht="14.4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="20" spans="3:4" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C20" s="34"/>
     </row>
-    <row r="21" spans="2:6" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="21" spans="3:4" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C21" s="34"/>
     </row>
-    <row r="22" spans="2:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C22" s="34"/>
-    </row>
-    <row r="23" spans="2:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C23" s="34"/>
-    </row>
-    <row r="24" spans="2:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C24" s="1"/>
+    <row r="22" spans="3:4" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C22" s="1"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="D4:D17">
+  <conditionalFormatting sqref="D4:D15">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"P"</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="C16" r:id="rId1" display="https://openclassrooms.com/fr/courses/8063076-initiez-vous-au-machine-learning-1/8300129-augmentez-la-robustesse-de-vos-modeles" xr:uid="{D13701F3-E1C3-49C1-AE40-B83A0D2BA363}"/>
-    <hyperlink ref="C17" r:id="rId2" display="https://scikit-learn.org/stable/modules/generated/sklearn.model_selection.GridSearchCV.html" xr:uid="{CFB2E0C7-62E1-4E88-9B14-90296AB7E783}"/>
+    <hyperlink ref="C14" r:id="rId1" display="https://openclassrooms.com/fr/courses/8063076-initiez-vous-au-machine-learning-1/8300129-augmentez-la-robustesse-de-vos-modeles" xr:uid="{D13701F3-E1C3-49C1-AE40-B83A0D2BA363}"/>
+    <hyperlink ref="C15" r:id="rId2" display="https://scikit-learn.org/stable/modules/generated/sklearn.model_selection.GridSearchCV.html" xr:uid="{CFB2E0C7-62E1-4E88-9B14-90296AB7E783}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <customProperties>
-    <customPr name="IbpWorksheetKeyString_GUID" r:id="rId3"/>
-  </customProperties>
 </worksheet>
 </file>
</xml_diff>